<commit_message>
fix: admin dashboard refetch + signature placement for new template
Rejected timesheets resubmitted by part-timers were staying visible as
'rejected' in the admin dashboard because the list page only fetched on
mount. The DB row correctly transitioned to 'submitted', but an
already-open admin tab never saw it. Refetch on focus / visibilitychange
so the list stays current without a manual reload.

Template gained explicit CASUAL WORKER SIGNATURE (B54) and HEAD OF CAFÉ
SIGNATURE (G54) placeholders. Move the signature image anchors to sit
below their labels (rows 55-58) and split columns B-F / G-J so each
signature lands under the correct heading.
</commit_message>
<xml_diff>
--- a/docs/RoundboyRoasters Timesheet.xlsx
+++ b/docs/RoundboyRoasters Timesheet.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nyanyk/Antigravity/CafeOS/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B62285D0-A650-F446-B885-8F682769FFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65BAC94-3398-DE44-BA9B-408141D78A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3520" yWindow="740" windowWidth="25220" windowHeight="17480" activeTab="1" xr2:uid="{B47A14C8-0129-5D48-96D8-6AFA4601A6B3}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{B47A14C8-0129-5D48-96D8-6AFA4601A6B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Timesheet" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Timesheet!$B$1:$H$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Timesheet!$B$1:$H$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="53">
   <si>
     <t>DATE</t>
   </si>
@@ -163,6 +163,7 @@
       <rPr>
         <sz val="10"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>:</t>
     </r>
@@ -200,13 +201,37 @@
   </si>
   <si>
     <t>BREAK (No of Hours)</t>
+  </si>
+  <si>
+    <t>Tue</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>Thu</t>
+  </si>
+  <si>
+    <t>Fri</t>
+  </si>
+  <si>
+    <t>Sat</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>CASUAL WORKER SIGNATURE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -245,44 +270,12 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -299,6 +292,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -308,7 +308,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -445,12 +445,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -500,71 +518,74 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -572,50 +593,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1333,14 +1360,14 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40" t="s">
+      <c r="C10" s="41"/>
+      <c r="D10" s="41" t="s">
         <v>4</v>
       </c>
       <c r="E10" s="11" t="s">
@@ -1349,24 +1376,24 @@
       <c r="F10" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="40" t="s">
+      <c r="G10" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40" t="s">
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="40"/>
+      <c r="A11" s="41"/>
       <c r="B11" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="40"/>
+      <c r="D11" s="41"/>
       <c r="E11" s="12" t="s">
         <v>5</v>
       </c>
@@ -1382,7 +1409,7 @@
       <c r="I11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="40"/>
+      <c r="J11" s="41"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="5">
@@ -1849,30 +1876,30 @@
       <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:10" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="41" t="s">
+      <c r="A43" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
     </row>
     <row r="45" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="B45" s="39"/>
-      <c r="C45" s="39"/>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
     </row>
     <row r="46" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="7"/>
@@ -1962,7 +1989,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC35BB4-89FE-8346-B982-8F509749680F}">
   <sheetPr published="0"/>
-  <dimension ref="B3:I69"/>
+  <dimension ref="B3:I58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="1"/>
@@ -1973,60 +2000,52 @@
     <col min="6" max="6" width="11.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="33.1640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.1640625" style="19"/>
-    <col min="10" max="16384" width="9.1640625" style="1"/>
+    <col min="9" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="43"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="15"/>
-      <c r="I3" s="1"/>
     </row>
     <row r="4" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="C4" s="19"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="42"/>
-      <c r="D5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="24"/>
       <c r="E5" s="7"/>
       <c r="F5" s="15"/>
-      <c r="I5" s="27"/>
+      <c r="I5" s="21"/>
     </row>
     <row r="6" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="I6" s="28"/>
+      <c r="I6" s="22"/>
     </row>
     <row r="7" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="38"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="25"/>
       <c r="E7" s="7"/>
       <c r="F7" s="15"/>
-      <c r="I7" s="27"/>
+      <c r="I7" s="21"/>
     </row>
     <row r="8" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="24"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="27"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="F8" s="3"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="21"/>
     </row>
     <row r="9" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="3"/>
@@ -2035,54 +2054,55 @@
       <c r="H9" s="14"/>
     </row>
     <row r="10" spans="2:9" s="13" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B10" s="46" t="s">
+      <c r="B10" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="49" t="s">
+      <c r="D10" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="50"/>
-      <c r="F10" s="46" t="s">
+      <c r="E10" s="32"/>
+      <c r="F10" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="G10" s="53" t="s">
+      <c r="G10" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="45" t="s">
+      <c r="H10" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="2:9" s="13" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="52"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="23"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="2:9" s="13" customFormat="1" ht="42" x14ac:dyDescent="0.15">
-      <c r="B12" s="48"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="22" t="s">
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="48"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="23"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B13" s="21"/>
-      <c r="C13" s="18"/>
+      <c r="B13" s="17">
+        <v>46266</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
@@ -2090,8 +2110,12 @@
       <c r="H13" s="6"/>
     </row>
     <row r="14" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B14" s="21"/>
-      <c r="C14" s="18"/>
+      <c r="B14" s="17">
+        <v>46267</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
@@ -2099,8 +2123,12 @@
       <c r="H14" s="6"/>
     </row>
     <row r="15" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="21"/>
-      <c r="C15" s="18"/>
+      <c r="B15" s="17">
+        <v>46268</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
@@ -2108,8 +2136,12 @@
       <c r="H15" s="6"/>
     </row>
     <row r="16" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="21"/>
-      <c r="C16" s="18"/>
+      <c r="B16" s="17">
+        <v>46269</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
@@ -2117,8 +2149,12 @@
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B17" s="21"/>
-      <c r="C17" s="18"/>
+      <c r="B17" s="17">
+        <v>46270</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -2126,8 +2162,12 @@
       <c r="H17" s="6"/>
     </row>
     <row r="18" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B18" s="21"/>
-      <c r="C18" s="18"/>
+      <c r="B18" s="17">
+        <v>46271</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -2135,8 +2175,12 @@
       <c r="H18" s="6"/>
     </row>
     <row r="19" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B19" s="21"/>
-      <c r="C19" s="18"/>
+      <c r="B19" s="17">
+        <v>46272</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -2144,8 +2188,12 @@
       <c r="H19" s="6"/>
     </row>
     <row r="20" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B20" s="21"/>
-      <c r="C20" s="18"/>
+      <c r="B20" s="17">
+        <v>46273</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -2153,8 +2201,12 @@
       <c r="H20" s="6"/>
     </row>
     <row r="21" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B21" s="21"/>
-      <c r="C21" s="18"/>
+      <c r="B21" s="17">
+        <v>46274</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -2162,8 +2214,12 @@
       <c r="H21" s="6"/>
     </row>
     <row r="22" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B22" s="21"/>
-      <c r="C22" s="18"/>
+      <c r="B22" s="17">
+        <v>46275</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -2171,8 +2227,12 @@
       <c r="H22" s="6"/>
     </row>
     <row r="23" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B23" s="21"/>
-      <c r="C23" s="18"/>
+      <c r="B23" s="17">
+        <v>46276</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
@@ -2182,8 +2242,12 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B24" s="21"/>
-      <c r="C24" s="18"/>
+      <c r="B24" s="17">
+        <v>46277</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
@@ -2191,8 +2255,12 @@
       <c r="H24" s="6"/>
     </row>
     <row r="25" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B25" s="21"/>
-      <c r="C25" s="18"/>
+      <c r="B25" s="17">
+        <v>46278</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -2200,8 +2268,12 @@
       <c r="H25" s="6"/>
     </row>
     <row r="26" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B26" s="21"/>
-      <c r="C26" s="18"/>
+      <c r="B26" s="17">
+        <v>46279</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -2209,8 +2281,12 @@
       <c r="H26" s="6"/>
     </row>
     <row r="27" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B27" s="21"/>
-      <c r="C27" s="18"/>
+      <c r="B27" s="17">
+        <v>46280</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -2218,8 +2294,12 @@
       <c r="H27" s="6"/>
     </row>
     <row r="28" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B28" s="21"/>
-      <c r="C28" s="18"/>
+      <c r="B28" s="17">
+        <v>46281</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
@@ -2227,8 +2307,12 @@
       <c r="H28" s="6"/>
     </row>
     <row r="29" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B29" s="21"/>
-      <c r="C29" s="18"/>
+      <c r="B29" s="17">
+        <v>46282</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
@@ -2236,8 +2320,12 @@
       <c r="H29" s="6"/>
     </row>
     <row r="30" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B30" s="21"/>
-      <c r="C30" s="18"/>
+      <c r="B30" s="17">
+        <v>46283</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
@@ -2245,8 +2333,12 @@
       <c r="H30" s="6"/>
     </row>
     <row r="31" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B31" s="21"/>
-      <c r="C31" s="18"/>
+      <c r="B31" s="17">
+        <v>46284</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
@@ -2254,127 +2346,170 @@
       <c r="H31" s="6"/>
     </row>
     <row r="32" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B32" s="21"/>
-      <c r="C32" s="18"/>
+      <c r="B32" s="17">
+        <v>46285</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="6"/>
     </row>
-    <row r="33" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B33" s="21"/>
-      <c r="C33" s="18"/>
+    <row r="33" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B33" s="17">
+        <v>46286</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
     </row>
-    <row r="34" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B34" s="21"/>
-      <c r="C34" s="18"/>
+    <row r="34" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B34" s="17">
+        <v>46287</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
     </row>
-    <row r="35" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="21"/>
-      <c r="C35" s="18"/>
+    <row r="35" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B35" s="17">
+        <v>46288</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
     </row>
-    <row r="36" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="21"/>
-      <c r="C36" s="18"/>
+    <row r="36" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B36" s="17">
+        <v>46289</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
     </row>
-    <row r="37" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B37" s="21"/>
-      <c r="C37" s="18"/>
+    <row r="37" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B37" s="17">
+        <v>46290</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
     </row>
-    <row r="38" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B38" s="21"/>
-      <c r="C38" s="18"/>
+    <row r="38" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B38" s="17">
+        <v>46291</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
     </row>
-    <row r="39" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B39" s="21"/>
-      <c r="C39" s="18"/>
+    <row r="39" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B39" s="17">
+        <v>46292</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
     </row>
-    <row r="40" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B40" s="21"/>
-      <c r="C40" s="18"/>
+    <row r="40" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B40" s="17">
+        <v>46293</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
     </row>
-    <row r="41" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B41" s="21"/>
-      <c r="C41" s="18"/>
+    <row r="41" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B41" s="17">
+        <v>46294</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
     </row>
-    <row r="42" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B42" s="21"/>
-      <c r="C42" s="18"/>
+    <row r="42" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B42" s="17">
+        <v>46295</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
     </row>
-    <row r="43" spans="2:9" ht="21" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B43" s="21"/>
-      <c r="C43" s="18"/>
+    <row r="43" spans="2:8" ht="21" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B43" s="17"/>
+      <c r="C43" s="5"/>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
     </row>
-    <row r="44" spans="2:9" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B44" s="41" t="s">
+    <row r="44" spans="2:8" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B44" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C44" s="41"/>
-      <c r="D44" s="41"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
+      <c r="C44" s="30"/>
+      <c r="D44" s="30"/>
+      <c r="E44" s="30"/>
+      <c r="F44" s="30"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
-      <c r="I44" s="24"/>
-    </row>
-    <row r="45" spans="2:9" ht="6" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="46" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="45" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="46" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B46" s="15" t="s">
         <v>34</v>
       </c>
@@ -2385,107 +2520,78 @@
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
-    <row r="48" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B48" s="16"/>
-      <c r="C48" s="16"/>
-    </row>
-    <row r="50" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-    </row>
-    <row r="51" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B51" s="30" t="s">
+    <row r="49" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B49" s="49"/>
+      <c r="C49" s="50"/>
+      <c r="D49" s="51"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="43"/>
+    </row>
+    <row r="50" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B50" s="52"/>
+      <c r="C50" s="53"/>
+      <c r="D50" s="54"/>
+      <c r="G50" s="44"/>
+      <c r="H50" s="45"/>
+    </row>
+    <row r="51" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B51" s="52"/>
+      <c r="C51" s="53"/>
+      <c r="D51" s="54"/>
+      <c r="G51" s="44"/>
+      <c r="H51" s="45"/>
+    </row>
+    <row r="52" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B52" s="52"/>
+      <c r="C52" s="53"/>
+      <c r="D52" s="54"/>
+      <c r="G52" s="44"/>
+      <c r="H52" s="45"/>
+    </row>
+    <row r="53" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B53" s="55"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="56"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="47"/>
+    </row>
+    <row r="54" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B54" s="57" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54" s="57"/>
+      <c r="D54" s="57"/>
+      <c r="E54" s="57"/>
+      <c r="F54" s="57"/>
+      <c r="G54" s="57" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B52" s="29"/>
-    </row>
-    <row r="53" spans="2:9" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="19"/>
-      <c r="F53" s="19"/>
-    </row>
-    <row r="54" spans="2:9" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B54" s="31"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-    </row>
-    <row r="55" spans="2:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C55" s="19"/>
-      <c r="D55" s="19"/>
-      <c r="E55" s="19"/>
-      <c r="F55" s="19"/>
-    </row>
-    <row r="56" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="57" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="59" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B59" s="32"/>
-      <c r="C59" s="44"/>
-      <c r="F59" s="19"/>
-    </row>
-    <row r="60" spans="2:9" s="17" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B60" s="33"/>
-      <c r="C60" s="44"/>
-      <c r="F60" s="20"/>
-      <c r="I60" s="20"/>
-    </row>
-    <row r="61" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B61" s="33"/>
-      <c r="C61" s="44"/>
-    </row>
-    <row r="62" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B62" s="33"/>
-      <c r="C62" s="44"/>
-    </row>
-    <row r="63" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B63" s="33"/>
-      <c r="C63" s="34"/>
-    </row>
-    <row r="64" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B64" s="33"/>
-      <c r="C64" s="44"/>
-    </row>
-    <row r="65" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B65" s="33"/>
-      <c r="C65" s="44"/>
-    </row>
-    <row r="66" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B66" s="35"/>
-      <c r="C66" s="44"/>
-    </row>
-    <row r="67" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B67" s="35"/>
-      <c r="C67" s="44"/>
-    </row>
-    <row r="68" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B68" s="35"/>
-      <c r="C68" s="44"/>
-    </row>
-    <row r="69" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B69" s="35"/>
-      <c r="C69" s="44"/>
-    </row>
+    <row r="55" spans="2:8" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B55" s="58"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+    </row>
+    <row r="56" spans="2:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="57" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="58" spans="2:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G10:G12"/>
-    <mergeCell ref="B10:B12"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="C64:C69"/>
+    <mergeCell ref="G49:H53"/>
+    <mergeCell ref="B49:D53"/>
     <mergeCell ref="H10:H12"/>
     <mergeCell ref="F10:F12"/>
     <mergeCell ref="C10:C12"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="D10:E11"/>
+    <mergeCell ref="G10:G12"/>
+    <mergeCell ref="B10:B12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>